<commit_message>
Fix: remove excessive freeze panes on Financial Reconciliation tab
</commit_message>
<xml_diff>
--- a/Barbourville_EV_Charging_Analysis.xlsx
+++ b/Barbourville_EV_Charging_Analysis.xlsx
@@ -1905,11 +1905,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="37609529"/>
-        <c:axId val="47371031"/>
+        <c:axId val="74447781"/>
+        <c:axId val="98713005"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="37609529"/>
+        <c:axId val="74447781"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1941,7 +1941,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47371031"/>
+        <c:crossAx val="98713005"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1949,7 +1949,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47371031"/>
+        <c:axId val="98713005"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2025,7 +2025,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37609529"/>
+        <c:crossAx val="74447781"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2304,11 +2304,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29439590"/>
-        <c:axId val="3508592"/>
+        <c:axId val="6819159"/>
+        <c:axId val="4958890"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29439590"/>
+        <c:axId val="6819159"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2340,7 +2340,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3508592"/>
+        <c:crossAx val="4958890"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2348,7 +2348,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3508592"/>
+        <c:axId val="4958890"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2424,7 +2424,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29439590"/>
+        <c:crossAx val="6819159"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2631,11 +2631,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86076098"/>
-        <c:axId val="11798268"/>
+        <c:axId val="64591316"/>
+        <c:axId val="79822019"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86076098"/>
+        <c:axId val="64591316"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2667,7 +2667,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11798268"/>
+        <c:crossAx val="79822019"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2675,7 +2675,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11798268"/>
+        <c:axId val="79822019"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2751,7 +2751,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86076098"/>
+        <c:crossAx val="64591316"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2987,11 +2987,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="95889530"/>
-        <c:axId val="66738216"/>
+        <c:axId val="27591221"/>
+        <c:axId val="91144380"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="95889530"/>
+        <c:axId val="27591221"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3023,7 +3023,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66738216"/>
+        <c:crossAx val="91144380"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3031,7 +3031,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66738216"/>
+        <c:axId val="91144380"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3107,7 +3107,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95889530"/>
+        <c:crossAx val="27591221"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3386,11 +3386,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57316210"/>
-        <c:axId val="74073659"/>
+        <c:axId val="86255926"/>
+        <c:axId val="83864939"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57316210"/>
+        <c:axId val="86255926"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3422,7 +3422,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74073659"/>
+        <c:crossAx val="83864939"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3430,7 +3430,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="74073659"/>
+        <c:axId val="83864939"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3506,7 +3506,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57316210"/>
+        <c:crossAx val="86255926"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3695,11 +3695,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="93432899"/>
-        <c:axId val="86534067"/>
+        <c:axId val="55233044"/>
+        <c:axId val="76683964"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93432899"/>
+        <c:axId val="55233044"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3731,7 +3731,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86534067"/>
+        <c:crossAx val="76683964"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3739,7 +3739,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86534067"/>
+        <c:axId val="76683964"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3815,7 +3815,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93432899"/>
+        <c:crossAx val="55233044"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4004,11 +4004,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="99293543"/>
-        <c:axId val="85518679"/>
+        <c:axId val="36552803"/>
+        <c:axId val="98532082"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="99293543"/>
+        <c:axId val="36552803"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4040,7 +4040,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85518679"/>
+        <c:crossAx val="98532082"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4048,7 +4048,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85518679"/>
+        <c:axId val="98532082"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4124,7 +4124,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99293543"/>
+        <c:crossAx val="36552803"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4316,11 +4316,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="78915233"/>
-        <c:axId val="1939195"/>
+        <c:axId val="15136659"/>
+        <c:axId val="9195601"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="78915233"/>
+        <c:axId val="15136659"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4352,7 +4352,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1939195"/>
+        <c:crossAx val="9195601"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4360,7 +4360,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1939195"/>
+        <c:axId val="9195601"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4436,7 +4436,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78915233"/>
+        <c:crossAx val="15136659"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4643,11 +4643,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="98376549"/>
-        <c:axId val="40193428"/>
+        <c:axId val="10422392"/>
+        <c:axId val="33256063"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="98376549"/>
+        <c:axId val="10422392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4679,7 +4679,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40193428"/>
+        <c:crossAx val="33256063"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4687,7 +4687,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40193428"/>
+        <c:axId val="33256063"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4763,7 +4763,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98376549"/>
+        <c:crossAx val="10422392"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4999,11 +4999,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="17859539"/>
-        <c:axId val="40977424"/>
+        <c:axId val="3932302"/>
+        <c:axId val="56391207"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="17859539"/>
+        <c:axId val="3932302"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5035,7 +5035,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40977424"/>
+        <c:crossAx val="56391207"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5043,7 +5043,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40977424"/>
+        <c:axId val="56391207"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5119,7 +5119,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17859539"/>
+        <c:crossAx val="3932302"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>